<commit_message>
assorted org stuff for updated data
</commit_message>
<xml_diff>
--- a/tables/hotel_treat_char.xlsx
+++ b/tables/hotel_treat_char.xlsx
@@ -1,82 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10308"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sam-heft-neal/Library/CloudStorage/GoogleDrive-sheftneal@gmail.com/.shortcut-targets-by-id/1-eKbXSB87cnTVZBZo_FVNT0VhouhJlaP/BEARLLC/Projects/California/CIty/Los Angeles /Living Wage/Updates/tables/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86A9DA59-0F6B-B04F-95E0-FD597C0449B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="660" windowWidth="29460" windowHeight="17340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
-  <si>
-    <t>Measure</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>Hotels</t>
-  </si>
-  <si>
-    <t>Total rooms</t>
-  </si>
-  <si>
-    <t>Average rooms</t>
-  </si>
-  <si>
-    <t>Average star rating</t>
-  </si>
-  <si>
-    <t>Share with restaurant</t>
-  </si>
-  <si>
-    <t>Average meeting rooms</t>
-  </si>
-  <si>
-    <t>Average neighborhood income</t>
-  </si>
-  <si>
-    <t>Median neighborhood home value</t>
-  </si>
-  <si>
-    <t>Share neighborhood pop Hispanic</t>
-  </si>
-  <si>
-    <t>Share neighborhood pop NH White</t>
-  </si>
-  <si>
-    <t>Share neighborhood pop NH Black</t>
-  </si>
-  <si>
-    <t>Share neighborhood pop NH Asian</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="172" formatCode="0.0"/>
-    <numFmt numFmtId="174" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-  </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -86,13 +25,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -117,39 +49,27 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="174" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Currency" xfId="1" builtinId="4"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -187,7 +107,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -221,7 +141,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -256,10 +175,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -432,156 +350,194 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.6640625" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>3</v>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Measure</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Hotels</t>
+        </is>
       </c>
       <c r="B2">
-        <v>313</v>
+        <v>342</v>
       </c>
       <c r="C2">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>4</v>
+        <v>135</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Total rooms</t>
+        </is>
       </c>
       <c r="B3">
-        <v>22600</v>
+        <v>24026</v>
       </c>
       <c r="C3">
-        <v>19195</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="2">
-        <v>72.204472843450631</v>
-      </c>
-      <c r="C4" s="2">
-        <v>156.05691056910581</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="2">
-        <v>2.4568690095846639</v>
-      </c>
-      <c r="C5" s="2">
-        <v>3.2926829268292681</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="2">
-        <v>10.22727272727273</v>
-      </c>
-      <c r="C6" s="2">
-        <v>4.9186046511627914</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="2">
-        <v>17.252396166134211</v>
-      </c>
-      <c r="C7" s="2">
-        <v>61.788617886178884</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="3">
-        <v>97133.773162939295</v>
-      </c>
-      <c r="C8" s="3">
-        <v>104517.42276422759</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="3">
-        <v>881024</v>
-      </c>
-      <c r="C9" s="3">
-        <v>924315</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" s="2">
-        <v>47.546246099485003</v>
-      </c>
-      <c r="C10" s="2">
-        <v>35.885489477052467</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" s="2">
-        <v>26.416614514335041</v>
-      </c>
-      <c r="C11" s="2">
-        <v>34.604830259313211</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="2">
-        <v>10.70917422417739</v>
-      </c>
-      <c r="C12" s="2">
-        <v>7.8291929418994419</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13" s="2">
-        <v>10.711260482472531</v>
-      </c>
-      <c r="C13" s="2">
-        <v>16.20514386021981</v>
+        <v>20389</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Average rooms</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>70.2514619883041</v>
+      </c>
+      <c r="C4">
+        <v>151.0296296296296</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Median rooms</t>
+        </is>
+      </c>
+      <c r="B5">
+        <v>26</v>
+      </c>
+      <c r="C5">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Average star rating</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>2.435672514619883</v>
+      </c>
+      <c r="C6">
+        <v>3.251851851851852</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Share with restaurant</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>16.95906432748539</v>
+      </c>
+      <c r="C7">
+        <v>57.77777777777779</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Average meeting rooms</t>
+        </is>
+      </c>
+      <c r="B8">
+        <v>11.71739130434782</v>
+      </c>
+      <c r="C8">
+        <v>4.208791208791209</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Average neighborhood income</t>
+        </is>
+      </c>
+      <c r="B9">
+        <v>102072.932748538</v>
+      </c>
+      <c r="C9">
+        <v>109730.6296296296</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Median neighborhood home value</t>
+        </is>
+      </c>
+      <c r="B10">
+        <v>886486.4298245615</v>
+      </c>
+      <c r="C10">
+        <v>945361.8740740741</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Share neighborhood pop Hispanic</t>
+        </is>
+      </c>
+      <c r="B11">
+        <v>47.94627539653261</v>
+      </c>
+      <c r="C11">
+        <v>35.43290478949375</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Share neighborhood pop NH White</t>
+        </is>
+      </c>
+      <c r="B12">
+        <v>26.10141469819032</v>
+      </c>
+      <c r="C12">
+        <v>34.98791059491537</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Share neighborhood pop NH Black</t>
+        </is>
+      </c>
+      <c r="B13">
+        <v>10.33497007842528</v>
+      </c>
+      <c r="C13">
+        <v>7.608768115325776</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Share neighborhood pop NH Asian</t>
+        </is>
+      </c>
+      <c r="B14">
+        <v>11.03818896619836</v>
+      </c>
+      <c r="C14">
+        <v>16.44820770844451</v>
       </c>
     </row>
   </sheetData>

</xml_diff>